<commit_message>
FIX: Sensitivity Analysis SH
</commit_message>
<xml_diff>
--- a/Sensitivity Analysis/SH/sensitivity_analysis_results.xlsx
+++ b/Sensitivity Analysis/SH/sensitivity_analysis_results.xlsx
@@ -34,7 +34,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -49,6 +49,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F9F9F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -78,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -87,6 +92,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -606,702 +617,728 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>gcn_depth_1</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F3" s="4" t="n">
         <v>1052192</v>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="G3" s="5" t="n">
         <v>0.1237208404654295</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="H3" s="5" t="n">
         <v>3707035.778365916</v>
       </c>
-      <c r="I3" s="3" t="n">
+      <c r="I3" s="5" t="n">
         <v>1353.356533280077</v>
       </c>
-      <c r="J3" s="3" t="n">
+      <c r="J3" s="5" t="n">
         <v>0.7216674334867839</v>
       </c>
-      <c r="K3" s="3" t="n">
-        <v>5.261057235999979</v>
-      </c>
-      <c r="L3" s="3" t="n">
-        <v>3.853899999873982</v>
-      </c>
-      <c r="M3" s="2" t="n"/>
-      <c r="N3" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="K3" s="5" t="n">
+        <v>5.299881774999958</v>
+      </c>
+      <c r="L3" s="5" t="n">
+        <v>3.85871999958334</v>
+      </c>
+      <c r="M3" s="5" t="n">
+        <v>106.88525390625</v>
+      </c>
+      <c r="N3" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>— (did not beat baseline)</t>
+          <t>Sensitivity_Analysis_SH\best_models\gcn_depth_1_best_model.pth</t>
         </is>
       </c>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="P3" s="4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>gcn_depth_2</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="4" t="n">
         <v>1056352</v>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="G4" s="5" t="n">
         <v>0.1259281665694957</v>
       </c>
-      <c r="H4" s="3" t="n">
+      <c r="H4" s="5" t="n">
         <v>3676973.531645881</v>
       </c>
-      <c r="I4" s="3" t="n">
+      <c r="I4" s="5" t="n">
         <v>1352.266151796965</v>
       </c>
-      <c r="J4" s="3" t="n">
+      <c r="J4" s="5" t="n">
         <v>0.7239245744438719</v>
       </c>
-      <c r="K4" s="3" t="n">
-        <v>4.814538921999993</v>
-      </c>
-      <c r="L4" s="3" t="n">
-        <v>3.908031579416466</v>
-      </c>
-      <c r="M4" s="2" t="n"/>
-      <c r="N4" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="K4" s="5" t="n">
+        <v>4.861796027000091</v>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>3.924012631116631</v>
+      </c>
+      <c r="M4" s="5" t="n">
+        <v>132.69677734375</v>
+      </c>
+      <c r="N4" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>— (did not beat baseline)</t>
+          <t>Sensitivity_Analysis_SH\best_models\gcn_depth_2_best_model.pth</t>
         </is>
       </c>
-      <c r="P4" s="2" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>gcn_depth_3</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="4" t="n">
         <v>1060512</v>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="G5" s="5" t="n">
         <v>0.1233143748677507</v>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="H5" s="5" t="n">
         <v>3637810.357925957</v>
       </c>
-      <c r="I5" s="3" t="n">
+      <c r="I5" s="5" t="n">
         <v>1343.176210172235</v>
       </c>
-      <c r="J5" s="3" t="n">
+      <c r="J5" s="5" t="n">
         <v>0.7268650334267293</v>
       </c>
-      <c r="K5" s="3" t="n">
-        <v>5.034922985000012</v>
-      </c>
-      <c r="L5" s="3" t="n">
-        <v>4.018797895083767</v>
-      </c>
-      <c r="M5" s="2" t="n"/>
-      <c r="N5" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="K5" s="5" t="n">
+        <v>5.072466153999994</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>3.987862104641911</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>140.31787109375</v>
+      </c>
+      <c r="N5" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>— (did not beat baseline)</t>
+          <t>Sensitivity_Analysis_SH\best_models\gcn_depth_3_best_model.pth</t>
         </is>
       </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="P5" s="4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>gcn_depth_7</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C6" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="4" t="n">
         <v>1077152</v>
       </c>
-      <c r="G6" s="3" t="n">
+      <c r="G6" s="5" t="n">
         <v>0.1246258095477004</v>
       </c>
-      <c r="H6" s="3" t="n">
+      <c r="H6" s="5" t="n">
         <v>3678071.667391337</v>
       </c>
-      <c r="I6" s="3" t="n">
+      <c r="I6" s="5" t="n">
         <v>1356.821576101612</v>
       </c>
-      <c r="J6" s="3" t="n">
+      <c r="J6" s="5" t="n">
         <v>0.7238421239473871</v>
       </c>
-      <c r="K6" s="3" t="n">
-        <v>6.00676832899997</v>
-      </c>
-      <c r="L6" s="3" t="n">
-        <v>4.528012631252702</v>
-      </c>
-      <c r="M6" s="2" t="n"/>
-      <c r="N6" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O6" s="2" t="inlineStr">
+      <c r="K6" s="5" t="n">
+        <v>5.963628527999972</v>
+      </c>
+      <c r="L6" s="5" t="n">
+        <v>4.406715789809823</v>
+      </c>
+      <c r="M6" s="5" t="n">
+        <v>140.2783203125</v>
+      </c>
+      <c r="N6" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>— (did not beat baseline)</t>
+          <t>Sensitivity_Analysis_SH\best_models\gcn_depth_7_best_model.pth</t>
         </is>
       </c>
-      <c r="P6" s="2" t="inlineStr">
+      <c r="P6" s="4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>hidden_32</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C7" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="4" t="n">
         <v>597824</v>
       </c>
-      <c r="G7" s="3" t="n">
+      <c r="G7" s="5" t="n">
         <v>0.1204620052357109</v>
       </c>
-      <c r="H7" s="3" t="n">
+      <c r="H7" s="5" t="n">
         <v>3607457.288543055</v>
       </c>
-      <c r="I7" s="3" t="n">
+      <c r="I7" s="5" t="n">
         <v>1345.825574130364</v>
       </c>
-      <c r="J7" s="3" t="n">
+      <c r="J7" s="5" t="n">
         <v>0.7291440100020836</v>
       </c>
-      <c r="K7" s="3" t="n">
-        <v>5.421040846999968</v>
-      </c>
-      <c r="L7" s="3" t="n">
-        <v>4.034646315956611</v>
-      </c>
-      <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="K7" s="5" t="n">
+        <v>5.383206562999985</v>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>3.959652631218839</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>93.1669921875</v>
+      </c>
+      <c r="N7" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>— (did not beat baseline)</t>
+          <t>Sensitivity_Analysis_SH\best_models\hidden_32_best_model.pth</t>
         </is>
       </c>
-      <c r="P7" s="2" t="inlineStr">
+      <c r="P7" s="4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>hidden_128</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C8" s="4" t="n">
         <v>128</v>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="4" t="n">
         <v>2053856</v>
       </c>
-      <c r="G8" s="3" t="n">
+      <c r="G8" s="5" t="n">
         <v>0.1223823945513185</v>
       </c>
-      <c r="H8" s="3" t="n">
+      <c r="H8" s="5" t="n">
         <v>3752388.553690132</v>
       </c>
-      <c r="I8" s="3" t="n">
+      <c r="I8" s="5" t="n">
         <v>1367.907794322092</v>
       </c>
-      <c r="J8" s="3" t="n">
+      <c r="J8" s="5" t="n">
         <v>0.7182622453231964</v>
       </c>
-      <c r="K8" s="3" t="n">
-        <v>5.766008874999971</v>
-      </c>
-      <c r="L8" s="3" t="n">
-        <v>4.332582104880681</v>
-      </c>
-      <c r="M8" s="2" t="n"/>
-      <c r="N8" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O8" s="2" t="inlineStr">
+      <c r="K8" s="5" t="n">
+        <v>5.715684869999968</v>
+      </c>
+      <c r="L8" s="5" t="n">
+        <v>4.289608420712236</v>
+      </c>
+      <c r="M8" s="5" t="n">
+        <v>220.00927734375</v>
+      </c>
+      <c r="N8" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>— (did not beat baseline)</t>
+          <t>Sensitivity_Analysis_SH\best_models\hidden_128_best_model.pth</t>
         </is>
       </c>
-      <c r="P8" s="2" t="inlineStr">
+      <c r="P8" s="4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>hidden_256</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="2" t="n">
+      <c r="C9" s="4" t="n">
         <v>256</v>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D9" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="F9" s="4" t="n">
         <v>4195936</v>
       </c>
-      <c r="G9" s="3" t="n">
-        <v>0.1241704729689779</v>
-      </c>
-      <c r="H9" s="3" t="n">
-        <v>3781015.79349661</v>
-      </c>
-      <c r="I9" s="3" t="n">
-        <v>1377.777470582528</v>
-      </c>
-      <c r="J9" s="3" t="n">
-        <v>0.7161128479059859</v>
-      </c>
-      <c r="K9" s="3" t="n">
-        <v>5.846929901999975</v>
-      </c>
-      <c r="L9" s="3" t="n">
-        <v>4.384006315146842</v>
-      </c>
-      <c r="M9" s="2" t="n"/>
-      <c r="N9" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O9" s="2" t="inlineStr">
+      <c r="G9" s="5" t="n">
+        <v>0.1239961820122387</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>3700755.774178034</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>1362.069950558416</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>0.7221389502963942</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>5.823963820999925</v>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>4.349013683263604</v>
+      </c>
+      <c r="M9" s="5" t="n">
+        <v>401.17041015625</v>
+      </c>
+      <c r="N9" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>— (did not beat baseline)</t>
+          <t>Sensitivity_Analysis_SH\best_models\hidden_256_best_model.pth</t>
         </is>
       </c>
-      <c r="P9" s="2" t="inlineStr">
+      <c r="P9" s="4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>kernel_3</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C10" s="2" t="n">
+      <c r="C10" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D10" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="F10" s="4" t="n">
         <v>1061920</v>
       </c>
-      <c r="G10" s="3" t="n">
+      <c r="G10" s="5" t="n">
         <v>0.1191238344323878</v>
       </c>
-      <c r="H10" s="3" t="n">
+      <c r="H10" s="5" t="n">
         <v>3464688.219259308</v>
       </c>
-      <c r="I10" s="3" t="n">
+      <c r="I10" s="5" t="n">
         <v>1318.351338767687</v>
       </c>
-      <c r="J10" s="3" t="n">
+      <c r="J10" s="5" t="n">
         <v>0.7398634321626016</v>
       </c>
-      <c r="K10" s="3" t="n">
-        <v>5.744651512000055</v>
-      </c>
-      <c r="L10" s="3" t="n">
-        <v>4.332028420666527</v>
-      </c>
-      <c r="M10" s="2" t="n"/>
-      <c r="N10" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O10" s="2" t="inlineStr">
+      <c r="K10" s="5" t="n">
+        <v>5.717670529999887</v>
+      </c>
+      <c r="L10" s="5" t="n">
+        <v>4.302254737367069</v>
+      </c>
+      <c r="M10" s="5" t="n">
+        <v>173.75390625</v>
+      </c>
+      <c r="N10" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>— (did not beat baseline)</t>
+          <t>Sensitivity_Analysis_SH\best_models\kernel_3_best_model.pth</t>
         </is>
       </c>
-      <c r="P10" s="2" t="inlineStr">
+      <c r="P10" s="4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>kernel_5</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="C11" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D11" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="F11" s="4" t="n">
         <v>1065376</v>
       </c>
-      <c r="G11" s="3" t="n">
+      <c r="G11" s="5" t="n">
         <v>0.1220613878353366</v>
       </c>
-      <c r="H11" s="3" t="n">
+      <c r="H11" s="5" t="n">
         <v>3562061.321282318</v>
       </c>
-      <c r="I11" s="3" t="n">
+      <c r="I11" s="5" t="n">
         <v>1333.561032830316</v>
       </c>
-      <c r="J11" s="3" t="n">
+      <c r="J11" s="5" t="n">
         <v>0.7325524411132073</v>
       </c>
-      <c r="K11" s="3" t="n">
-        <v>4.64685381000003</v>
-      </c>
-      <c r="L11" s="3" t="n">
-        <v>4.329473684590898</v>
-      </c>
-      <c r="M11" s="2" t="n"/>
-      <c r="N11" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O11" s="2" t="inlineStr">
+      <c r="K11" s="5" t="n">
+        <v>4.613773405999964</v>
+      </c>
+      <c r="L11" s="5" t="n">
+        <v>4.247812630522898</v>
+      </c>
+      <c r="M11" s="5" t="n">
+        <v>141.47216796875</v>
+      </c>
+      <c r="N11" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>— (did not beat baseline)</t>
+          <t>Sensitivity_Analysis_SH\best_models\kernel_5_best_model.pth</t>
         </is>
       </c>
-      <c r="P11" s="2" t="inlineStr">
+      <c r="P11" s="4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>kernel_11</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B12" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C12" s="2" t="n">
+      <c r="C12" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D12" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E12" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="F12" s="4" t="n">
         <v>1075744</v>
       </c>
-      <c r="G12" s="3" t="n">
+      <c r="G12" s="5" t="n">
         <v>0.1179972133428163</v>
       </c>
-      <c r="H12" s="3" t="n">
+      <c r="H12" s="5" t="n">
         <v>3899360.20474407</v>
       </c>
-      <c r="I12" s="3" t="n">
+      <c r="I12" s="5" t="n">
         <v>1389.892521068709</v>
       </c>
-      <c r="J12" s="3" t="n">
+      <c r="J12" s="5" t="n">
         <v>0.7072272838908685</v>
       </c>
-      <c r="K12" s="3" t="n">
-        <v>5.396334897000052</v>
-      </c>
-      <c r="L12" s="3" t="n">
-        <v>4.320817894002079</v>
-      </c>
-      <c r="M12" s="2" t="n"/>
-      <c r="N12" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
+      <c r="K12" s="5" t="n">
+        <v>5.375890566000017</v>
+      </c>
+      <c r="L12" s="5" t="n">
+        <v>4.281769475384959</v>
+      </c>
+      <c r="M12" s="5" t="n">
+        <v>147.72412109375</v>
+      </c>
+      <c r="N12" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>— (did not beat baseline)</t>
+          <t>Sensitivity_Analysis_SH\best_models\kernel_11_best_model.pth</t>
         </is>
       </c>
-      <c r="P12" s="2" t="inlineStr">
+      <c r="P12" s="4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>dilation_1</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B13" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C13" s="2" t="n">
+      <c r="C13" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="D13" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="F13" s="4" t="n">
         <v>1068832</v>
       </c>
-      <c r="G13" s="3" t="n">
+      <c r="G13" s="5" t="n">
         <v>0.1210614009570254</v>
       </c>
-      <c r="H13" s="3" t="n">
+      <c r="H13" s="5" t="n">
         <v>3534166.515824856</v>
       </c>
-      <c r="I13" s="3" t="n">
+      <c r="I13" s="5" t="n">
         <v>1332.150523665938</v>
       </c>
-      <c r="J13" s="3" t="n">
+      <c r="J13" s="5" t="n">
         <v>0.7346468457155779</v>
       </c>
-      <c r="K13" s="3" t="n">
-        <v>5.055226407000009</v>
-      </c>
-      <c r="L13" s="3" t="n">
-        <v>4.412422105087899</v>
-      </c>
-      <c r="M13" s="2" t="n"/>
-      <c r="N13" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O13" s="2" t="inlineStr">
+      <c r="K13" s="5" t="n">
+        <v>5.042284816000029</v>
+      </c>
+      <c r="L13" s="5" t="n">
+        <v>4.409419999482404</v>
+      </c>
+      <c r="M13" s="5" t="n">
+        <v>137.638671875</v>
+      </c>
+      <c r="N13" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>— (did not beat baseline)</t>
+          <t>Sensitivity_Analysis_SH\best_models\dilation_1_best_model.pth</t>
         </is>
       </c>
-      <c r="P13" s="2" t="inlineStr">
+      <c r="P13" s="4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>dilation_2</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B14" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C14" s="2" t="n">
+      <c r="C14" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D14" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="F14" s="4" t="n">
         <v>1068832</v>
       </c>
-      <c r="G14" s="3" t="n">
+      <c r="G14" s="5" t="n">
         <v>0.118768530175546</v>
       </c>
-      <c r="H14" s="3" t="n">
+      <c r="H14" s="5" t="n">
         <v>3494941.999768865</v>
       </c>
-      <c r="I14" s="3" t="n">
+      <c r="I14" s="5" t="n">
         <v>1321.13537547432</v>
       </c>
-      <c r="J14" s="3" t="n">
+      <c r="J14" s="5" t="n">
         <v>0.7375919104187072</v>
       </c>
-      <c r="K14" s="3" t="n">
-        <v>5.750425558999996</v>
-      </c>
-      <c r="L14" s="3" t="n">
-        <v>4.367069473894509</v>
-      </c>
-      <c r="M14" s="2" t="n"/>
-      <c r="N14" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O14" s="2" t="inlineStr">
+      <c r="K14" s="5" t="n">
+        <v>5.739268483000051</v>
+      </c>
+      <c r="L14" s="5" t="n">
+        <v>4.450307368288601</v>
+      </c>
+      <c r="M14" s="5" t="n">
+        <v>140.2783203125</v>
+      </c>
+      <c r="N14" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>— (did not beat baseline)</t>
+          <t>Sensitivity_Analysis_SH\best_models\dilation_2_best_model.pth</t>
         </is>
       </c>
-      <c r="P14" s="2" t="inlineStr">
+      <c r="P14" s="4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>dilation_5</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B15" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C15" s="2" t="n">
+      <c r="C15" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D15" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="F15" s="4" t="n">
         <v>1068832</v>
       </c>
-      <c r="G15" s="3" t="n">
+      <c r="G15" s="5" t="n">
         <v>0.1209732741497609</v>
       </c>
-      <c r="H15" s="3" t="n">
+      <c r="H15" s="5" t="n">
         <v>3808461.209542298</v>
       </c>
-      <c r="I15" s="3" t="n">
+      <c r="I15" s="5" t="n">
         <v>1372.239586049188</v>
       </c>
-      <c r="J15" s="3" t="n">
+      <c r="J15" s="5" t="n">
         <v>0.7140521844692855</v>
       </c>
-      <c r="K15" s="3" t="n">
-        <v>5.416456913000002</v>
-      </c>
-      <c r="L15" s="3" t="n">
-        <v>4.303508421090603</v>
-      </c>
-      <c r="M15" s="2" t="n"/>
-      <c r="N15" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O15" s="2" t="inlineStr">
+      <c r="K15" s="5" t="n">
+        <v>5.655586276999966</v>
+      </c>
+      <c r="L15" s="5" t="n">
+        <v>4.542538946445443</v>
+      </c>
+      <c r="M15" s="5" t="n">
+        <v>146.0283203125</v>
+      </c>
+      <c r="N15" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>— (did not beat baseline)</t>
+          <t>Sensitivity_Analysis_SH\best_models\dilation_5_best_model.pth</t>
         </is>
       </c>
-      <c r="P15" s="2" t="inlineStr">
+      <c r="P15" s="4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -1592,10 +1629,10 @@
         <v>0.255278887303204</v>
       </c>
       <c r="N3" t="n">
-        <v>0.5713088960472634</v>
+        <v>0.5713088486992052</v>
       </c>
       <c r="O3" t="n">
-        <v>0.2648607173896566</v>
+        <v>0.2648548954071439</v>
       </c>
       <c r="P3" t="n">
         <v>0.5690468242550872</v>
@@ -1675,10 +1712,10 @@
         <v>0.2255384579909091</v>
       </c>
       <c r="N4" t="n">
-        <v>0.5070206006232382</v>
+        <v>0.5076660507775004</v>
       </c>
       <c r="O4" t="n">
-        <v>0.2305884080349791</v>
+        <v>0.2306711355946502</v>
       </c>
       <c r="P4" t="n">
         <v>0.5013717160188297</v>
@@ -1758,10 +1795,10 @@
         <v>0.2119465790574952</v>
       </c>
       <c r="N5" t="n">
-        <v>0.4708208623294537</v>
+        <v>0.4713522289393298</v>
       </c>
       <c r="O5" t="n">
-        <v>0.2255297931557407</v>
+        <v>0.2255125611792413</v>
       </c>
       <c r="P5" t="n">
         <v>0.4700847331167488</v>
@@ -1841,10 +1878,10 @@
         <v>0.1965832882465757</v>
       </c>
       <c r="N6" t="n">
-        <v>0.447007017636055</v>
+        <v>0.4468322224889599</v>
       </c>
       <c r="O6" t="n">
-        <v>0.2044801190875623</v>
+        <v>0.2024525204027185</v>
       </c>
       <c r="P6" t="n">
         <v>0.4475080320554382</v>
@@ -1924,10 +1961,10 @@
         <v>0.1876649387674976</v>
       </c>
       <c r="N7" t="n">
-        <v>0.43008067786897</v>
+        <v>0.4313112223209374</v>
       </c>
       <c r="O7" t="n">
-        <v>0.1883864470244366</v>
+        <v>0.1896428356935479</v>
       </c>
       <c r="P7" t="n">
         <v>0.4313461731725178</v>
@@ -2007,10 +2044,10 @@
         <v>0.1794813832610237</v>
       </c>
       <c r="N8" t="n">
-        <v>0.4151002554661585</v>
+        <v>0.4154826846139016</v>
       </c>
       <c r="O8" t="n">
-        <v>0.1856048994374518</v>
+        <v>0.1834277919284543</v>
       </c>
       <c r="P8" t="n">
         <v>0.4172409799827244</v>
@@ -2090,10 +2127,10 @@
         <v>0.1753495182005727</v>
       </c>
       <c r="N9" t="n">
-        <v>0.4039671742977136</v>
+        <v>0.4041991233317112</v>
       </c>
       <c r="O9" t="n">
-        <v>0.182599204763466</v>
+        <v>0.1795302884729237</v>
       </c>
       <c r="P9" t="n">
         <v>0.4086140129244775</v>
@@ -2173,10 +2210,10 @@
         <v>0.1702893836689847</v>
       </c>
       <c r="N10" t="n">
-        <v>0.3952424084774057</v>
+        <v>0.3944112833449458</v>
       </c>
       <c r="O10" t="n">
-        <v>0.1748925623274883</v>
+        <v>0.1763401687601391</v>
       </c>
       <c r="P10" t="n">
         <v>0.3973006682387798</v>
@@ -2256,10 +2293,10 @@
         <v>0.1675158723124436</v>
       </c>
       <c r="N11" t="n">
-        <v>0.3848523335855569</v>
+        <v>0.3864499776029749</v>
       </c>
       <c r="O11" t="n">
-        <v>0.1711962483823299</v>
+        <v>0.170266555261095</v>
       </c>
       <c r="P11" t="n">
         <v>0.388913014795593</v>
@@ -2339,10 +2376,10 @@
         <v>0.1637119138233211</v>
       </c>
       <c r="N12" t="n">
-        <v>0.3771014109813313</v>
+        <v>0.3787607380757966</v>
       </c>
       <c r="O12" t="n">
-        <v>0.1667274425034316</v>
+        <v>0.1683557179699443</v>
       </c>
       <c r="P12" t="n">
         <v>0.3823455735379925</v>
@@ -2422,10 +2459,10 @@
         <v>0.1615276216738382</v>
       </c>
       <c r="N13" t="n">
-        <v>0.3696264556446987</v>
+        <v>0.3714006775068341</v>
       </c>
       <c r="O13" t="n">
-        <v>0.1645063898165007</v>
+        <v>0.1638931496334927</v>
       </c>
       <c r="P13" t="n">
         <v>0.3751818707575164</v>
@@ -2505,10 +2542,10 @@
         <v>0.157445515620009</v>
       </c>
       <c r="N14" t="n">
-        <v>0.3641657619244409</v>
+        <v>0.3644596495420859</v>
       </c>
       <c r="O14" t="n">
-        <v>0.1593265243786938</v>
+        <v>0.160777279308864</v>
       </c>
       <c r="P14" t="n">
         <v>0.3688680624697396</v>
@@ -2588,10 +2625,10 @@
         <v>0.1534385312234565</v>
       </c>
       <c r="N15" t="n">
-        <v>0.3573210767308193</v>
+        <v>0.3587299230867685</v>
       </c>
       <c r="O15" t="n">
-        <v>0.1574175238267196</v>
+        <v>0.1578406429830558</v>
       </c>
       <c r="P15" t="n">
         <v>0.3640287340501063</v>
@@ -2671,10 +2708,10 @@
         <v>0.1504114221743479</v>
       </c>
       <c r="N16" t="n">
-        <v>0.3532429979828031</v>
+        <v>0.3533374564944681</v>
       </c>
       <c r="O16" t="n">
-        <v>0.1545797183311411</v>
+        <v>0.155155466299276</v>
       </c>
       <c r="P16" t="n">
         <v>0.3588146760093474</v>
@@ -2754,10 +2791,10 @@
         <v>0.1471838857978582</v>
       </c>
       <c r="N17" t="n">
-        <v>0.3489794146282274</v>
+        <v>0.3473803335896124</v>
       </c>
       <c r="O17" t="n">
-        <v>0.1501730951119442</v>
+        <v>0.1504592261638264</v>
       </c>
       <c r="P17" t="n">
         <v>0.3544061235295221</v>
@@ -2837,10 +2874,10 @@
         <v>0.1449408452501711</v>
       </c>
       <c r="N18" t="n">
-        <v>0.3433572426184046</v>
+        <v>0.3426422441677022</v>
       </c>
       <c r="O18" t="n">
-        <v>0.1512657055935385</v>
+        <v>0.1497293200571926</v>
       </c>
       <c r="P18" t="n">
         <v>0.3496790095502606</v>
@@ -2920,10 +2957,10 @@
         <v>0.142896113442067</v>
       </c>
       <c r="N19" t="n">
-        <v>0.34034500797454</v>
+        <v>0.3394668038184325</v>
       </c>
       <c r="O19" t="n">
-        <v>0.1489405930232333</v>
+        <v>0.1480229957675447</v>
       </c>
       <c r="P19" t="n">
         <v>0.3470917037932946</v>
@@ -3003,10 +3040,10 @@
         <v>0.1418835899070361</v>
       </c>
       <c r="N20" t="n">
-        <v>0.3366141797841206</v>
+        <v>0.3353565274245096</v>
       </c>
       <c r="O20" t="n">
-        <v>0.1458661863010149</v>
+        <v>0.1452796647363171</v>
       </c>
       <c r="P20" t="n">
         <v>0.3422692852927556</v>
@@ -3086,10 +3123,10 @@
         <v>0.1406809221573022</v>
       </c>
       <c r="N21" t="n">
-        <v>0.3329204743022398</v>
+        <v>0.3315530341538146</v>
       </c>
       <c r="O21" t="n">
-        <v>0.1446533975362474</v>
+        <v>0.1437655114663803</v>
       </c>
       <c r="P21" t="n">
         <v>0.3381402305368678</v>
@@ -3169,10 +3206,10 @@
         <v>0.1394441268805947</v>
       </c>
       <c r="N22" t="n">
-        <v>0.3294588830894171</v>
+        <v>0.3282759462708906</v>
       </c>
       <c r="O22" t="n">
-        <v>0.1446146229662153</v>
+        <v>0.1429686756728559</v>
       </c>
       <c r="P22" t="n">
         <v>0.3356302415653301</v>
@@ -3252,10 +3289,10 @@
         <v>0.1407392124683425</v>
       </c>
       <c r="N23" t="n">
-        <v>0.3268745431466721</v>
+        <v>0.3261858922375347</v>
       </c>
       <c r="O23" t="n">
-        <v>0.1431564388378542</v>
+        <v>0.1424115482831792</v>
       </c>
       <c r="P23" t="n">
         <v>0.3323557373301568</v>
@@ -3335,10 +3372,10 @@
         <v>0.1399298565443225</v>
       </c>
       <c r="N24" t="n">
-        <v>0.3245511083472711</v>
+        <v>0.3243315413390817</v>
       </c>
       <c r="O24" t="n">
-        <v>0.1426187257415482</v>
+        <v>0.140909926680734</v>
       </c>
       <c r="P24" t="n">
         <v>0.3302308525445111</v>
@@ -3418,10 +3455,10 @@
         <v>0.1399766945432187</v>
       </c>
       <c r="N25" t="n">
-        <v>0.3213387352411251</v>
+        <v>0.3206436670172337</v>
       </c>
       <c r="O25" t="n">
-        <v>0.1415207456911401</v>
+        <v>0.1399250504351696</v>
       </c>
       <c r="P25" t="n">
         <v>0.3272708754592381</v>
@@ -3501,10 +3538,10 @@
         <v>0.1385652028993532</v>
       </c>
       <c r="N26" t="n">
-        <v>0.3186420694044426</v>
+        <v>0.3188010073257388</v>
       </c>
       <c r="O26" t="n">
-        <v>0.1420401375436661</v>
+        <v>0.1413289017937317</v>
       </c>
       <c r="P26" t="n">
         <v>0.3246962734253333</v>
@@ -3584,10 +3621,10 @@
         <v>0.1393911658729217</v>
       </c>
       <c r="N27" t="n">
-        <v>0.3182349034645451</v>
+        <v>0.3177764295717962</v>
       </c>
       <c r="O27" t="n">
-        <v>0.1421569909672348</v>
+        <v>0.1395251357699839</v>
       </c>
       <c r="P27" t="n">
         <v>0.3219374435550117</v>
@@ -3667,10 +3704,10 @@
         <v>0.1384018969494013</v>
       </c>
       <c r="N28" t="n">
-        <v>0.3150250336009081</v>
+        <v>0.3152756518573078</v>
       </c>
       <c r="O28" t="n">
-        <v>0.1402513048782641</v>
+        <v>0.1394217295039977</v>
       </c>
       <c r="P28" t="n">
         <v>0.319672887439207</v>
@@ -3750,10 +3787,10 @@
         <v>0.1373070035205812</v>
       </c>
       <c r="N29" t="n">
-        <v>0.3138778637395377</v>
+        <v>0.3136689955870853</v>
       </c>
       <c r="O29" t="n">
-        <v>0.1408056961942692</v>
+        <v>0.1404009323795231</v>
       </c>
       <c r="P29" t="n">
         <v>0.3174308261773692</v>
@@ -3833,10 +3870,10 @@
         <v>0.1377121524467152</v>
       </c>
       <c r="N30" t="n">
-        <v>0.311482467749013</v>
+        <v>0.3113194557841321</v>
       </c>
       <c r="O30" t="n">
-        <v>0.1405327861596431</v>
+        <v>0.1391390570800523</v>
       </c>
       <c r="P30" t="n">
         <v>0.3149433943853037</v>
@@ -3916,10 +3953,10 @@
         <v>0.1374062600412539</v>
       </c>
       <c r="N31" t="n">
-        <v>0.3091624924855834</v>
+        <v>0.3094068778863132</v>
       </c>
       <c r="O31" t="n">
-        <v>0.1405953005602469</v>
+        <v>0.1395950720892573</v>
       </c>
       <c r="P31" t="n">
         <v>0.3128468961845893</v>
@@ -3999,10 +4036,10 @@
         <v>0.1350498938438844</v>
       </c>
       <c r="N32" t="n">
-        <v>0.3082350213271359</v>
+        <v>0.3083435040692014</v>
       </c>
       <c r="O32" t="n">
-        <v>0.1385155709992562</v>
+        <v>0.1379652763716877</v>
       </c>
       <c r="P32" t="n">
         <v>0.3115338308819325</v>
@@ -4082,10 +4119,10 @@
         <v>0.1374345292071147</v>
       </c>
       <c r="N33" t="n">
-        <v>0.3060775526351082</v>
+        <v>0.3061021671156834</v>
       </c>
       <c r="O33" t="n">
-        <v>0.1392438022267758</v>
+        <v>0.1385330312923357</v>
       </c>
       <c r="P33" t="n">
         <v>0.3092082173344218</v>
@@ -4165,10 +4202,10 @@
         <v>0.1396525886993171</v>
       </c>
       <c r="N34" t="n">
-        <v>0.3047765323275592</v>
+        <v>0.3048737730080764</v>
       </c>
       <c r="O34" t="n">
-        <v>0.1398651236193064</v>
+        <v>0.1383899961389145</v>
       </c>
       <c r="P34" t="n">
         <v>0.3069332374240758</v>
@@ -4248,10 +4285,10 @@
         <v>0.1376248760414975</v>
       </c>
       <c r="N35" t="n">
-        <v>0.3038573874853577</v>
+        <v>0.3037045376801247</v>
       </c>
       <c r="O35" t="n">
-        <v>0.1398306242855532</v>
+        <v>0.1399067082746449</v>
       </c>
       <c r="P35" t="n">
         <v>0.3064544791095086</v>
@@ -4331,10 +4368,10 @@
         <v>0.1357867184703295</v>
       </c>
       <c r="N36" t="n">
-        <v>0.3029503324434619</v>
+        <v>0.3025641614259713</v>
       </c>
       <c r="O36" t="n">
-        <v>0.1386728131649446</v>
+        <v>0.1382836077210246</v>
       </c>
       <c r="P36" t="n">
         <v>0.3048223319619182</v>
@@ -4414,10 +4451,10 @@
         <v>0.130643544290975</v>
       </c>
       <c r="N37" t="n">
-        <v>0.2969449574935151</v>
+        <v>0.2975930559350362</v>
       </c>
       <c r="O37" t="n">
-        <v>0.1311082503739364</v>
+        <v>0.1298662323067535</v>
       </c>
       <c r="P37" t="n">
         <v>0.3035827157796446</v>
@@ -4497,10 +4534,10 @@
         <v>0.1301199457399091</v>
       </c>
       <c r="N38" t="n">
-        <v>0.294063902450503</v>
+        <v>0.2941549071984893</v>
       </c>
       <c r="O38" t="n">
-        <v>0.1315001828824075</v>
+        <v>0.1305642125234768</v>
       </c>
       <c r="P38" t="n">
         <v>0.3023123082549092</v>
@@ -4580,10 +4617,10 @@
         <v>0.1299063908031248</v>
       </c>
       <c r="N39" t="n">
-        <v>0.2931524172882985</v>
+        <v>0.2936314194377372</v>
       </c>
       <c r="O39" t="n">
-        <v>0.1302736813145481</v>
+        <v>0.1299828041763026</v>
       </c>
       <c r="P39" t="n">
         <v>0.3004344787969931</v>
@@ -4663,10 +4700,10 @@
         <v>0.1301363441827042</v>
       </c>
       <c r="N40" t="n">
-        <v>0.2919376758992062</v>
+        <v>0.2924958631752294</v>
       </c>
       <c r="O40" t="n">
-        <v>0.1300392378387707</v>
+        <v>0.1299173665537062</v>
       </c>
       <c r="P40" t="n">
         <v>0.29918533070299</v>
@@ -4746,10 +4783,10 @@
         <v>0.1292674996110858</v>
       </c>
       <c r="N41" t="n">
-        <v>0.2919127861540065</v>
+        <v>0.292476850768405</v>
       </c>
       <c r="O41" t="n">
-        <v>0.1305665302527498</v>
+        <v>0.1300840741973751</v>
       </c>
       <c r="P41" t="n">
         <v>0.2977491378682465</v>
@@ -4829,10 +4866,10 @@
         <v>0.1293587828416149</v>
       </c>
       <c r="N42" t="n">
-        <v>0.2906675854691466</v>
+        <v>0.2881572408023141</v>
       </c>
       <c r="O42" t="n">
-        <v>0.1309000973361639</v>
+        <v>0.126392709556967</v>
       </c>
       <c r="P42" t="n">
         <v>0.2977119514356294</v>
@@ -4912,10 +4949,10 @@
         <v>0.1299159493848529</v>
       </c>
       <c r="N43" t="n">
-        <v>0.289712432810064</v>
+        <v>0.2877312324966587</v>
       </c>
       <c r="O43" t="n">
-        <v>0.1311185287444719</v>
+        <v>0.1264105105620562</v>
       </c>
       <c r="P43" t="n">
         <v>0.2927332749342349</v>
@@ -4995,10 +5032,10 @@
         <v>0.129610833740432</v>
       </c>
       <c r="N44" t="n">
-        <v>0.2895138058747855</v>
+        <v>0.2871965440466949</v>
       </c>
       <c r="O44" t="n">
-        <v>0.1308880233376914</v>
+        <v>0.1261783486745339</v>
       </c>
       <c r="P44" t="n">
         <v>0.2884709712486625</v>
@@ -5078,10 +5115,10 @@
         <v>0.1301377827434667</v>
       </c>
       <c r="N45" t="n">
-        <v>0.2868138419483302</v>
+        <v>0.2872984931127203</v>
       </c>
       <c r="O45" t="n">
-        <v>0.1270216885307918</v>
+        <v>0.1261828856599726</v>
       </c>
       <c r="P45" t="n">
         <v>0.2882135365501606</v>
@@ -5161,10 +5198,10 @@
         <v>0.1261508176768465</v>
       </c>
       <c r="N46" t="n">
-        <v>0.2856348936061404</v>
+        <v>0.2865898594158501</v>
       </c>
       <c r="O46" t="n">
-        <v>0.127008893051926</v>
+        <v>0.126335471868515</v>
       </c>
       <c r="P46" t="n">
         <v>0.287513788802225</v>
@@ -5244,10 +5281,10 @@
         <v>0.1257475372308827</v>
       </c>
       <c r="N47" t="n">
-        <v>0.2853774348521802</v>
+        <v>0.2866694017634457</v>
       </c>
       <c r="O47" t="n">
-        <v>0.1265631602145731</v>
+        <v>0.1262434675852407</v>
       </c>
       <c r="P47" t="n">
         <v>0.2866429447771746</v>
@@ -5327,10 +5364,10 @@
         <v>0.1258614167704114</v>
       </c>
       <c r="N48" t="n">
-        <v>0.2848488796286209</v>
+        <v>0.2857961548371526</v>
       </c>
       <c r="O48" t="n">
-        <v>0.126792253327689</v>
+        <v>0.126280167054537</v>
       </c>
       <c r="P48" t="n">
         <v>0.2857305864730386</v>
@@ -5410,10 +5447,10 @@
         <v>0.1254754965668734</v>
       </c>
       <c r="N49" t="n">
-        <v>0.2845302880471477</v>
+        <v>0.2843267456612489</v>
       </c>
       <c r="O49" t="n">
-        <v>0.1265629817997771</v>
+        <v>0.1253662447977279</v>
       </c>
       <c r="P49" t="n">
         <v>0.2853145357793508</v>
@@ -5493,10 +5530,10 @@
         <v>0.125491888376371</v>
       </c>
       <c r="N50" t="n">
-        <v>0.2838286565228941</v>
+        <v>0.283673000925637</v>
       </c>
       <c r="O50" t="n">
-        <v>0.1265675421443065</v>
+        <v>0.1252289127216351</v>
       </c>
       <c r="P50" t="n">
         <v>0.2854607081097955</v>
@@ -5576,10 +5613,10 @@
         <v>0.125565448823404</v>
       </c>
       <c r="N51" t="n">
-        <v>0.2842376465836076</v>
+        <v>0.2839728715629301</v>
       </c>
       <c r="O51" t="n">
-        <v>0.1267774846708896</v>
+        <v>0.1251262788166653</v>
       </c>
       <c r="P51" t="n">
         <v>0.2847625306035065</v>
@@ -5659,10 +5696,10 @@
         <v>0.1252140484997356</v>
       </c>
       <c r="N52" t="n">
-        <v>0.2818294481307573</v>
+        <v>0.2836683726656559</v>
       </c>
       <c r="O52" t="n">
-        <v>0.1258889824646164</v>
+        <v>0.1249655600143026</v>
       </c>
       <c r="P52" t="n">
         <v>0.2838993733144864</v>
@@ -5742,10 +5779,10 @@
         <v>0.1254572975354231</v>
       </c>
       <c r="N53" t="n">
-        <v>0.2810357751852416</v>
+        <v>0.2829306567589984</v>
       </c>
       <c r="O53" t="n">
-        <v>0.1258427965340718</v>
+        <v>0.1251695084442594</v>
       </c>
       <c r="P53" t="n">
         <v>0.283610598066561</v>
@@ -5825,10 +5862,10 @@
         <v>0.1256588499574941</v>
       </c>
       <c r="N54" t="n">
-        <v>0.2805936689974912</v>
+        <v>0.2821997999636386</v>
       </c>
       <c r="O54" t="n">
-        <v>0.125575613658115</v>
+        <v>0.1250022317339875</v>
       </c>
       <c r="P54" t="n">
         <v>0.2832191355602733</v>
@@ -5908,10 +5945,10 @@
         <v>0.1252912119677176</v>
       </c>
       <c r="N55" t="n">
-        <v>0.2809679433957709</v>
+        <v>0.2825283118787479</v>
       </c>
       <c r="O55" t="n">
-        <v>0.1255168953758417</v>
+        <v>0.1250197319408917</v>
       </c>
       <c r="P55" t="n">
         <v>0.2823947442778141</v>
@@ -5991,10 +6028,10 @@
         <v>0.1251785321047111</v>
       </c>
       <c r="N56" t="n">
-        <v>0.2810112676827981</v>
+        <v>0.2827150140199238</v>
       </c>
       <c r="O56" t="n">
-        <v>0.1253125418015585</v>
+        <v>0.1248448101366509</v>
       </c>
       <c r="P56" t="n">
         <v>0.2819248214618338</v>
@@ -6074,10 +6111,10 @@
         <v>0.1252909665737225</v>
       </c>
       <c r="N57" t="n">
-        <v>0.28073192502248</v>
+        <v>0.2827356721404876</v>
       </c>
       <c r="O57" t="n">
-        <v>0.1252956453197617</v>
+        <v>0.1247889536375902</v>
       </c>
       <c r="P57" t="n">
         <v>0.2812047125231284</v>
@@ -6157,10 +6194,10 @@
         <v>0.1251965602004559</v>
       </c>
       <c r="N58" t="n">
-        <v>0.2799964116396758</v>
+        <v>0.2818574775455348</v>
       </c>
       <c r="O58" t="n">
-        <v>0.1253982061444192</v>
+        <v>0.124916755328221</v>
       </c>
       <c r="P58" t="n">
         <v>0.2810343856646746</v>
@@ -6240,10 +6277,10 @@
         <v>0.1249171996071022</v>
       </c>
       <c r="N59" t="n">
-        <v>0.2799670673372803</v>
+        <v>0.2819590980485844</v>
       </c>
       <c r="O59" t="n">
-        <v>0.1252572590732301</v>
+        <v>0.1247799388627161</v>
       </c>
       <c r="P59" t="n">
         <v>0.281365955877833</v>
@@ -6323,10 +6360,10 @@
         <v>0.1253307035991124</v>
       </c>
       <c r="N60" t="n">
-        <v>0.2798228198503471</v>
+        <v>0.2815614873130167</v>
       </c>
       <c r="O60" t="n">
-        <v>0.1252772281212466</v>
+        <v>0.1246973166945485</v>
       </c>
       <c r="P60" t="n">
         <v>0.2807508183725865</v>
@@ -6406,10 +6443,10 @@
         <v>0.1253918193147651</v>
       </c>
       <c r="N61" t="n">
-        <v>0.279811334233642</v>
+        <v>0.2814839117915557</v>
       </c>
       <c r="O61" t="n">
-        <v>0.1252709384532455</v>
+        <v>0.1248966586795084</v>
       </c>
       <c r="P61" t="n">
         <v>0.2797932739245607</v>
@@ -6489,10 +6526,10 @@
         <v>0.125335024850329</v>
       </c>
       <c r="N62" t="n">
-        <v>0.2797859257703755</v>
+        <v>0.2820433503074044</v>
       </c>
       <c r="O62" t="n">
-        <v>0.1249133786091543</v>
+        <v>0.1245803620229114</v>
       </c>
       <c r="P62" t="n">
         <v>0.2791944804757122</v>
@@ -6572,10 +6609,10 @@
         <v>0.1251681328047903</v>
       </c>
       <c r="N63" t="n">
-        <v>0.2793124989692262</v>
+        <v>0.28090494443939</v>
       </c>
       <c r="O63" t="n">
-        <v>0.1249302133195558</v>
+        <v>0.1245907097389655</v>
       </c>
       <c r="P63" t="n">
         <v>0.2787748014255595</v>
@@ -6655,10 +6692,10 @@
         <v>0.1239052282418219</v>
       </c>
       <c r="N64" t="n">
-        <v>0.2792273957676448</v>
+        <v>0.2814295909815681</v>
       </c>
       <c r="O64" t="n">
-        <v>0.1249679534753062</v>
+        <v>0.1245994170728539</v>
       </c>
       <c r="P64" t="n">
         <v>0.2755008994414131</v>
@@ -6738,10 +6775,10 @@
         <v>0.1234726927490259</v>
       </c>
       <c r="N65" t="n">
-        <v>0.2791204702477813</v>
+        <v>0.2810830384899732</v>
       </c>
       <c r="O65" t="n">
-        <v>0.1250391070997076</v>
+        <v>0.1244713293236433</v>
       </c>
       <c r="P65" t="n">
         <v>0.2744342446734067</v>
@@ -6821,10 +6858,10 @@
         <v>0.1234325374837737</v>
       </c>
       <c r="N66" t="n">
-        <v>0.2789859491505314</v>
+        <v>0.2806314959257536</v>
       </c>
       <c r="O66" t="n">
-        <v>0.1248779883703255</v>
+        <v>0.1244784495128053</v>
       </c>
       <c r="P66" t="n">
         <v>0.2742817574800485</v>
@@ -6904,10 +6941,10 @@
         <v>0.1233653098401823</v>
       </c>
       <c r="N67" t="n">
-        <v>0.2790710200832159</v>
+        <v>0.280740338711405</v>
       </c>
       <c r="O67" t="n">
-        <v>0.1249812207355791</v>
+        <v>0.1245859861278868</v>
       </c>
       <c r="P67" t="n">
         <v>0.2742312259641524</v>
@@ -6987,10 +7024,10 @@
         <v>0.1234403158328971</v>
       </c>
       <c r="N68" t="n">
-        <v>0.2783342159445376</v>
+        <v>0.2804307779964734</v>
       </c>
       <c r="O68" t="n">
-        <v>0.1248543407977084</v>
+        <v>0.1245487409605816</v>
       </c>
       <c r="P68" t="n">
         <v>0.2741320792064325</v>
@@ -7070,10 +7107,10 @@
         <v>0.1233428564701914</v>
       </c>
       <c r="N69" t="n">
-        <v>0.2784044652566975</v>
+        <v>0.2800321269259111</v>
       </c>
       <c r="O69" t="n">
-        <v>0.1247659427189857</v>
+        <v>0.1244840046048773</v>
       </c>
       <c r="P69" t="n">
         <v>0.2736778077971406</v>
@@ -7153,10 +7190,10 @@
         <v>0.1233731741180681</v>
       </c>
       <c r="N70" t="n">
-        <v>0.2784583168581077</v>
+        <v>0.2789782062935748</v>
       </c>
       <c r="O70" t="n">
-        <v>0.1248175352431682</v>
+        <v>0.1242842137509463</v>
       </c>
       <c r="P70" t="n">
         <v>0.2713139405022709</v>
@@ -7236,10 +7273,10 @@
         <v>0.1232405683424856</v>
       </c>
       <c r="N71" t="n">
-        <v>0.2777558225413638</v>
+        <v>0.2784251822953338</v>
       </c>
       <c r="O71" t="n">
-        <v>0.1248813057223297</v>
+        <v>0.1243115784410311</v>
       </c>
       <c r="P71" t="n">
         <v>0.2717955209594538</v>
@@ -7319,10 +7356,10 @@
         <v>0.1232958765016222</v>
       </c>
       <c r="N72" t="n">
-        <v>0.2777011308552055</v>
+        <v>0.2787570524134327</v>
       </c>
       <c r="O72" t="n">
-        <v>0.1248271174500791</v>
+        <v>0.124231093059465</v>
       </c>
       <c r="P72" t="n">
         <v>0.2712707292708114</v>
@@ -7402,10 +7439,10 @@
         <v>0.1232942431899054</v>
       </c>
       <c r="N73" t="n">
-        <v>0.2778007725806773</v>
+        <v>0.2787875693812712</v>
       </c>
       <c r="O73" t="n">
-        <v>0.1247982609903022</v>
+        <v>0.1241328473278911</v>
       </c>
       <c r="P73" t="n">
         <v>0.2707409874977919</v>
@@ -7485,10 +7522,10 @@
         <v>0.1232726844122671</v>
       </c>
       <c r="N74" t="n">
-        <v>0.276588581222723</v>
+        <v>0.2786605613935523</v>
       </c>
       <c r="O74" t="n">
-        <v>0.1245769969548802</v>
+        <v>0.1241357577109367</v>
       </c>
       <c r="P74" t="n">
         <v>0.2703572622795968</v>
@@ -7568,10 +7605,10 @@
         <v>0.1232000531685748</v>
       </c>
       <c r="N75" t="n">
-        <v>0.276565831752157</v>
+        <v>0.2785271086790456</v>
       </c>
       <c r="O75" t="n">
-        <v>0.1246337608187174</v>
+        <v>0.1242261618014653</v>
       </c>
       <c r="P75" t="n">
         <v>0.2703402572320996</v>
@@ -7651,10 +7688,10 @@
         <v>0.1233162234480284</v>
       </c>
       <c r="N76" t="n">
-        <v>0.2766587821188233</v>
+        <v>0.2786080417169239</v>
       </c>
       <c r="O76" t="n">
-        <v>0.1246034576443537</v>
+        <v>0.124193276421224</v>
       </c>
       <c r="P76" t="n">
         <v>0.2705803414609652</v>
@@ -7734,10 +7771,10 @@
         <v>0.1234061759326379</v>
       </c>
       <c r="N77" t="n">
-        <v>0.2763628794878416</v>
+        <v>0.278632277413033</v>
       </c>
       <c r="O77" t="n">
-        <v>0.1245674513926616</v>
+        <v>0.1241783853620291</v>
       </c>
       <c r="P77" t="n">
         <v>0.270623129204475</v>
@@ -7817,10 +7854,10 @@
         <v>0.1232997100534184</v>
       </c>
       <c r="N78" t="n">
-        <v>0.2758360641909948</v>
+        <v>0.277621132521906</v>
       </c>
       <c r="O78" t="n">
-        <v>0.1244828541459022</v>
+        <v>0.1241878270722774</v>
       </c>
       <c r="P78" t="n">
         <v>0.2702329724315083</v>
@@ -7900,10 +7937,10 @@
         <v>0.1231376577206716</v>
       </c>
       <c r="N79" t="n">
-        <v>0.2756526721164635</v>
+        <v>0.2774219660425349</v>
       </c>
       <c r="O79" t="n">
-        <v>0.1244890872978282</v>
+        <v>0.1241378696939471</v>
       </c>
       <c r="P79" t="n">
         <v>0.2699771012869304</v>
@@ -7983,10 +8020,10 @@
         <v>0.123137943798258</v>
       </c>
       <c r="N80" t="n">
-        <v>0.2761551020698743</v>
+        <v>0.2780812188423534</v>
       </c>
       <c r="O80" t="n">
-        <v>0.1245546858016478</v>
+        <v>0.1242079914889622</v>
       </c>
       <c r="P80" t="n">
         <v>0.2700843229483012</v>
@@ -8066,10 +8103,10 @@
         <v>0.1233186184865784</v>
       </c>
       <c r="N81" t="n">
-        <v>0.276235298619132</v>
+        <v>0.2780878111058941</v>
       </c>
       <c r="O81" t="n">
-        <v>0.1244753342102833</v>
+        <v>0.1241744610347918</v>
       </c>
       <c r="P81" t="n">
         <v>0.2698582754098515</v>
@@ -8149,10 +8186,10 @@
         <v>0.1232090502008035</v>
       </c>
       <c r="N82" t="n">
-        <v>0.276115903599067</v>
+        <v>0.2777155909318566</v>
       </c>
       <c r="O82" t="n">
-        <v>0.1244584445518498</v>
+        <v>0.1241838022952481</v>
       </c>
       <c r="P82" t="n">
         <v>0.2692165542584637</v>
@@ -8232,10 +8269,10 @@
         <v>0.1230899342335761</v>
       </c>
       <c r="N83" t="n">
-        <v>0.2757617076000663</v>
+        <v>0.2773004443775672</v>
       </c>
       <c r="O83" t="n">
-        <v>0.1243563540355892</v>
+        <v>0.1241513404006861</v>
       </c>
       <c r="P83" t="n">
         <v>0.2698748590545443</v>
@@ -8309,10 +8346,10 @@
         <v>0.1230056828971268</v>
       </c>
       <c r="N84" t="n">
-        <v>0.2757779972138258</v>
+        <v>0.2773354592583692</v>
       </c>
       <c r="O84" t="n">
-        <v>0.1242737281326281</v>
+        <v>0.124106453665133</v>
       </c>
       <c r="P84" t="n">
         <v>0.2697881731767297</v>
@@ -8386,10 +8423,10 @@
         <v>0.1232788336406253</v>
       </c>
       <c r="N85" t="n">
-        <v>0.2757126837968826</v>
+        <v>0.2778566717186072</v>
       </c>
       <c r="O85" t="n">
-        <v>0.124287950293142</v>
+        <v>0.1240754376773779</v>
       </c>
       <c r="P85" t="n">
         <v>0.2696209025057509</v>
@@ -8463,10 +8500,10 @@
         <v>0.1231313810151603</v>
       </c>
       <c r="N86" t="n">
-        <v>0.2755504808429972</v>
+        <v>0.2773046236955672</v>
       </c>
       <c r="O86" t="n">
-        <v>0.1242799643731239</v>
+        <v>0.1240865349465487</v>
       </c>
       <c r="P86" t="n">
         <v>0.269779127205598</v>
@@ -8540,10 +8577,10 @@
         <v>0.1230261239926426</v>
       </c>
       <c r="N87" t="n">
-        <v>0.2755842261753798</v>
+        <v>0.2771322347045759</v>
       </c>
       <c r="O87" t="n">
-        <v>0.1243179190941915</v>
+        <v>0.1240829343109259</v>
       </c>
       <c r="P87" t="n">
         <v>0.2692280958435234</v>
@@ -8617,10 +8654,10 @@
         <v>0.1230378288357538</v>
       </c>
       <c r="N88" t="n">
-        <v>0.2750374843388694</v>
+        <v>0.2773386187622572</v>
       </c>
       <c r="O88" t="n">
-        <v>0.1242859348730773</v>
+        <v>0.1240960508014779</v>
       </c>
       <c r="P88" t="n">
         <v>0.2684171543084721</v>
@@ -8694,10 +8731,10 @@
         <v>0.1229714112242266</v>
       </c>
       <c r="N89" t="n">
-        <v>0.2745737269164759</v>
+        <v>0.2770250601878345</v>
       </c>
       <c r="O89" t="n">
-        <v>0.1243376960996918</v>
+        <v>0.124068301095038</v>
       </c>
       <c r="P89" t="n">
         <v>0.26871865291034</v>
@@ -8771,10 +8808,10 @@
         <v>0.1227386648652657</v>
       </c>
       <c r="N90" t="n">
-        <v>0.274371234121583</v>
+        <v>0.2768794315463447</v>
       </c>
       <c r="O90" t="n">
-        <v>0.124222844934129</v>
+        <v>0.1240591421932438</v>
       </c>
       <c r="P90" t="n">
         <v>0.2677553963335708</v>
@@ -8842,10 +8879,10 @@
         <v>0.1227591201111826</v>
       </c>
       <c r="N91" t="n">
-        <v>0.2747605328063509</v>
+        <v>0.2768805341814158</v>
       </c>
       <c r="O91" t="n">
-        <v>0.124182796124749</v>
+        <v>0.1240411504095762</v>
       </c>
       <c r="P91" t="n">
         <v>0.2683264836414682</v>
@@ -8907,10 +8944,10 @@
         <v>0.1227114675091389</v>
       </c>
       <c r="N92" t="n">
-        <v>0.2741931686273207</v>
+        <v>0.2768420231983116</v>
       </c>
       <c r="O92" t="n">
-        <v>0.1242310594273161</v>
+        <v>0.1240404134103078</v>
       </c>
       <c r="P92" t="n">
         <v>0.2678528278557514</v>
@@ -8972,10 +9009,10 @@
         <v>0.1225963034857141</v>
       </c>
       <c r="N93" t="n">
-        <v>0.2736128455237724</v>
+        <v>0.2762856664511124</v>
       </c>
       <c r="O93" t="n">
-        <v>0.1241731554535883</v>
+        <v>0.1240265773115109</v>
       </c>
       <c r="P93" t="n">
         <v>0.267825780620754</v>
@@ -9037,10 +9074,10 @@
         <v>0.1226352291675855</v>
       </c>
       <c r="N94" t="n">
-        <v>0.2750684164540759</v>
+        <v>0.2774934262647564</v>
       </c>
       <c r="O94" t="n">
-        <v>0.1242757434766664</v>
+        <v>0.1240601532009183</v>
       </c>
       <c r="P94" t="n">
         <v>0.2675084978748914</v>
@@ -9096,10 +9133,10 @@
         <v>0.1226391252415369</v>
       </c>
       <c r="N95" t="n">
-        <v>0.2739406353682788</v>
+        <v>0.2766786010192116</v>
       </c>
       <c r="O95" t="n">
-        <v>0.1241704729689779</v>
+        <v>0.1240321297616679</v>
       </c>
       <c r="P95" t="n">
         <v>0.2677410256893155</v>
@@ -9155,10 +9192,10 @@
         <v>0.1225963649435007</v>
       </c>
       <c r="N96" t="n">
-        <v>0.2736651542447126</v>
+        <v>0.2766791032341153</v>
       </c>
       <c r="O96" t="n">
-        <v>0.1242101187057489</v>
+        <v>0.1240347310691616</v>
       </c>
       <c r="P96" t="n">
         <v>0.2675798837184499</v>
@@ -9202,10 +9239,10 @@
         <v>0.1224886819777288</v>
       </c>
       <c r="N97" t="n">
-        <v>0.2736935778028322</v>
+        <v>0.2764447267348449</v>
       </c>
       <c r="O97" t="n">
-        <v>0.1242152705256428</v>
+        <v>0.124030220293801</v>
       </c>
       <c r="P97" t="n">
         <v>0.2669286426830617</v>
@@ -9243,10 +9280,10 @@
         <v>0.1223823945513185</v>
       </c>
       <c r="N98" t="n">
-        <v>0.2742138145930124</v>
+        <v>0.2771021532778447</v>
       </c>
       <c r="O98" t="n">
-        <v>0.1242543699942073</v>
+        <v>0.1240288450819801</v>
       </c>
       <c r="P98" t="n">
         <v>0.2667812215793662</v>
@@ -9284,10 +9321,10 @@
         <v>0.1224655289373988</v>
       </c>
       <c r="N99" t="n">
-        <v>0.2732060089097088</v>
+        <v>0.2763143922281753</v>
       </c>
       <c r="O99" t="n">
-        <v>0.1242672240133492</v>
+        <v>0.1240353604911694</v>
       </c>
       <c r="P99" t="n">
         <v>0.2667729927309544</v>
@@ -9325,10 +9362,10 @@
         <v>0.1225050223173992</v>
       </c>
       <c r="N100" t="n">
-        <v>0.2740488862269161</v>
+        <v>0.2770474690931242</v>
       </c>
       <c r="O100" t="n">
-        <v>0.1242890935771319</v>
+        <v>0.1240226374558952</v>
       </c>
       <c r="P100" t="n">
         <v>0.2670878710244296</v>
@@ -9366,10 +9403,10 @@
         <v>0.1225443962790376</v>
       </c>
       <c r="N101" t="n">
-        <v>0.2734051184544384</v>
+        <v>0.2764870239097511</v>
       </c>
       <c r="O101" t="n">
-        <v>0.1242659547347195</v>
+        <v>0.1239961820122387</v>
       </c>
       <c r="P101" t="n">
         <v>0.266700287575201</v>

</xml_diff>